<commit_message>
Round 3: fix contrast issue and CSV total-row format violation
RunSchedule_Owl512.xlsx: route numbers in gold #B8862B failed
contrast (~2.9:1) against the alternating cream fill on rows
8/10/12. Changed to the workbook's dark navy body-text color across
all six rows for consistency. Verified no formula cached values
were disturbed.

medical_billing_ledger.csv: removed the trailing TOTAL row, which
violated "every row after header is a data record." Confirmed it's
not a Must-match artifact for the billed/paid canonical values
(that's A15) and the remaining 81 line items independently foot to
the same $2,840,000/$196,000/$2,644,000 totals.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PxihHDWnbH3FCTMLDXxDWe
</commit_message>
<xml_diff>
--- a/filesystem/ACTD/Ops/RunSchedule_Owl512.xlsx
+++ b/filesystem/ACTD/Ops/RunSchedule_Owl512.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -126,6 +126,12 @@
       <color rgb="002E6B3B"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Helvetica"/>
+      <b val="1"/>
+      <color rgb="000E1B2C"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -180,7 +186,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="31">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -515,11 +521,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <top style="hair">
+        <color rgb="00C9C2B3"/>
+      </top>
+      <bottom style="hair">
+        <color rgb="00C9C2B3"/>
+      </bottom>
+    </border>
+    <border>
+      <right/>
+      <bottom style="medium">
+        <color rgb="00B8862B"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00B8862B"/>
+      </left>
+      <right/>
+      <bottom style="medium">
+        <color rgb="00B8862B"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -682,6 +712,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1009,7 +1054,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="62" t="inlineStr">
         <is>
           <t>ALDER CREEK TRANSIT DISTRICT — OPERATIONS</t>
         </is>
@@ -1157,7 +1202,7 @@
       <c r="N8" s="56" t="n"/>
     </row>
     <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="63" t="inlineStr">
         <is>
           <t>Block Assignment Header</t>
         </is>
@@ -1182,7 +1227,7 @@
           <t>Block ID:</t>
         </is>
       </c>
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="64" t="inlineStr">
         <is>
           <t>512-OWL</t>
         </is>
@@ -1214,7 +1259,7 @@
           <t>Operator Badge:</t>
         </is>
       </c>
-      <c r="B12" s="26" t="inlineStr">
+      <c r="B12" s="64" t="inlineStr">
         <is>
           <t>4417</t>
         </is>
@@ -1246,7 +1291,7 @@
           <t>Vehicle #:</t>
         </is>
       </c>
-      <c r="B13" s="26" t="inlineStr">
+      <c r="B13" s="64" t="inlineStr">
         <is>
           <t>4177</t>
         </is>
@@ -1278,7 +1323,7 @@
           <t>Scheduled Pullout:</t>
         </is>
       </c>
-      <c r="B14" s="26" t="inlineStr">
+      <c r="B14" s="64" t="inlineStr">
         <is>
           <t>10/17/2025 22:15</t>
         </is>
@@ -1310,7 +1355,7 @@
           <t>Sign / Bid Cycle:</t>
         </is>
       </c>
-      <c r="B15" s="26" t="inlineStr">
+      <c r="B15" s="64" t="inlineStr">
         <is>
           <t>Fall 2025 Sign</t>
         </is>
@@ -1337,7 +1382,7 @@
       <c r="N15" s="56" t="n"/>
     </row>
     <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="25" t="inlineStr">
+      <c r="A17" s="63" t="inlineStr">
         <is>
           <t>Block Manifest — Trip Roster</t>
         </is>
@@ -2293,7 +2338,7 @@
       </c>
     </row>
     <row r="32" ht="26" customHeight="1">
-      <c r="A32" s="25" t="inlineStr">
+      <c r="A32" s="63" t="inlineStr">
         <is>
           <t>Key Timepoint — S. Main / Third (Downtown Rivergate)</t>
         </is>
@@ -2377,7 +2422,7 @@
       <c r="N35" s="56" t="n"/>
     </row>
     <row r="37" ht="26" customHeight="1">
-      <c r="A37" s="25" t="inlineStr">
+      <c r="A37" s="63" t="inlineStr">
         <is>
           <t>Assignment Sign-Off</t>
         </is>
@@ -2618,7 +2663,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="62" t="inlineStr">
         <is>
           <t>ALDER CREEK TRANSIT DISTRICT — AUTHORIZED OWL ROUTES</t>
         </is>
@@ -2682,7 +2727,7 @@
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="42" t="inlineStr">
+      <c r="A7" s="65" t="inlineStr">
         <is>
           <t>510</t>
         </is>
@@ -2714,7 +2759,7 @@
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="45" t="inlineStr">
+      <c r="A8" s="66" t="inlineStr">
         <is>
           <t>511</t>
         </is>
@@ -2746,7 +2791,7 @@
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="42" t="inlineStr">
+      <c r="A9" s="65" t="inlineStr">
         <is>
           <t>512</t>
         </is>
@@ -2778,7 +2823,7 @@
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="45" t="inlineStr">
+      <c r="A10" s="66" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -2810,7 +2855,7 @@
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="42" t="inlineStr">
+      <c r="A11" s="65" t="inlineStr">
         <is>
           <t>517</t>
         </is>
@@ -2842,7 +2887,7 @@
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="45" t="inlineStr">
+      <c r="A12" s="66" t="inlineStr">
         <is>
           <t>519</t>
         </is>
@@ -2910,7 +2955,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="62" t="inlineStr">
         <is>
           <t>ALDER CREEK TRANSIT DISTRICT — SCHEDULE NOTES</t>
         </is>

</xml_diff>